<commit_message>
feat: integrar Lay 0x2 Zebra e Lay 2x0 Zebra no Portfolio e Resultados Forward + atualizar chaves de multiselect
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-12.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-12.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/21df80ec97692de0/Documentos/GitHub/ARKAD_PROD/metodos_aprovados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_6405B28954FABB4DC39B3211595ED87656CD4A47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE7AFF9A-5086-4114-919F-5DF9967A556B}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_6405B28954FABB4DC39B3211595ED87656CD4A47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19133D7E-E825-4D5A-82C1-DBE5916E256D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -629,6 +629,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -918,6 +922,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="18.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">

</xml_diff>